<commit_message>
updating task-3 Interactive Dashboarding
</commit_message>
<xml_diff>
--- a/Dashboard.xlsx
+++ b/Dashboard.xlsx
@@ -184,40 +184,40 @@
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1440,6 +1440,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-2439-4EFD-A353-A3F32B1F110C}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -1482,6 +1487,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-2439-4EFD-A353-A3F32B1F110C}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -1524,6 +1534,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-2439-4EFD-A353-A3F32B1F110C}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:cat>
             <c:strRef>

</xml_diff>